<commit_message>
fix(projects/pifil) Add missing document (blank form v0.3)
</commit_message>
<xml_diff>
--- a/projects/pifil/doc/dolphinfree-doc-24-002-protocole-2025-02-05.xlsx
+++ b/projects/pifil/doc/dolphinfree-doc-24-002-protocole-2025-02-05.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Engin" sheetId="1" state="visible" r:id="rId2"/>
@@ -1432,168 +1432,172 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1677,201 +1681,201 @@
   <dimension ref="A1:O28"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="0" t="n">
+      <c r="O2" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="O4" s="0" t="n">
+      <c r="C4" s="2"/>
+      <c r="O4" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O5" s="0" t="n">
+      <c r="O5" s="1" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="O6" s="0" t="n">
+      <c r="B6" s="3"/>
+      <c r="O6" s="1" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8" t="s">
+    <row r="11" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8"/>
+      <c r="B11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
-    </row>
-    <row r="12" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7"/>
-      <c r="B12" s="11" t="s">
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+    </row>
+    <row r="12" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8"/>
+      <c r="B12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-    </row>
-    <row r="13" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7"/>
-      <c r="B13" s="11" t="s">
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+    </row>
+    <row r="13" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8"/>
+      <c r="B13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-    </row>
-    <row r="14" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7"/>
-      <c r="B14" s="11" t="s">
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+    </row>
+    <row r="14" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8"/>
+      <c r="B14" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7"/>
-      <c r="B15" s="11" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+    </row>
+    <row r="15" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8"/>
+      <c r="B15" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10"/>
-    </row>
-    <row r="16" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="11" t="s">
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+    </row>
+    <row r="16" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8"/>
+      <c r="B16" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10"/>
-    </row>
-    <row r="17" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="11" t="s">
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+    </row>
+    <row r="17" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8"/>
+      <c r="B17" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="10" t="s">
+      <c r="C17" s="13"/>
+      <c r="D17" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="13" t="s">
+    <row r="18" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8"/>
+      <c r="B18" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="18" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18"/>
+      <c r="A24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18"/>
+      <c r="A25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18"/>
+      <c r="A26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18"/>
+      <c r="A27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18"/>
+      <c r="A28" s="19"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1903,324 +1907,325 @@
   <dimension ref="A1:Y42"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="53.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="69.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="27.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="26.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="33.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="26.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="25.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="22.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="53.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="69.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="29.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="27.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="34.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="26.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="33.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="25.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="22.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1"/>
+      <c r="B6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="7"/>
+      <c r="D12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="22" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="G14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="S14" s="23"/>
-      <c r="Y14" s="23"/>
+      <c r="B14" s="3"/>
+      <c r="G14" s="24"/>
+      <c r="M14" s="24"/>
+      <c r="S14" s="24"/>
+      <c r="Y14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="S15" s="23"/>
-      <c r="Y15" s="23"/>
+      <c r="A15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="M15" s="24"/>
+      <c r="S15" s="24"/>
+      <c r="Y15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="Y16" s="23"/>
+      <c r="G16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="Y16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="S17" s="23"/>
-      <c r="Y17" s="23"/>
+      <c r="G17" s="24"/>
+      <c r="M17" s="24"/>
+      <c r="S17" s="24"/>
+      <c r="Y17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="M18" s="23"/>
-      <c r="S18" s="23"/>
-      <c r="Y18" s="23"/>
+      <c r="A18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="M18" s="24"/>
+      <c r="S18" s="24"/>
+      <c r="Y18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="S19" s="23"/>
-      <c r="Y19" s="23"/>
+      <c r="G19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="S19" s="24"/>
+      <c r="Y19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="S25" s="23"/>
-      <c r="Y25" s="23"/>
+      <c r="G25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="S25" s="24"/>
+      <c r="Y25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="5" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="27" t="s">
+      <c r="D35" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G35" s="23"/>
-      <c r="M35" s="23"/>
-      <c r="S35" s="23"/>
-      <c r="Y35" s="23"/>
+      <c r="G35" s="24"/>
+      <c r="M35" s="24"/>
+      <c r="S35" s="24"/>
+      <c r="Y35" s="24"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2" t="s">
+      <c r="D36" s="3"/>
+      <c r="E36" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2" t="s">
+      <c r="D37" s="3"/>
+      <c r="E37" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="17" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="28" t="s">
+      <c r="B39" s="29" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="3" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2242,217 +2247,217 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="35.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="38.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="35.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="38.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1"/>
+      <c r="B7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="32" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="35" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="27" t="s">
+      <c r="C19" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="E19" s="31" t="s">
+      <c r="D19" s="32" t="s">
         <v>97</v>
       </c>
+      <c r="F19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="35"/>
+      <c r="B22" s="36"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="D26" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36" t="s">
+    <row r="27" s="2" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="2" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-    </row>
-    <row r="29" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" s="2" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
+    <row r="30" s="2" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="37" t="s">
+    <row r="31" s="2" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="38" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2474,35 +2479,35 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="15.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="15.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38"/>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="39"/>
+      <c r="B2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39"/>
-      <c r="B3" s="0" t="s">
+      <c r="A3" s="40"/>
+      <c r="B3" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="40"/>
-      <c r="B4" s="0" t="s">
+      <c r="A4" s="41"/>
+      <c r="B4" s="1" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>